<commit_message>
added pdf_scrapper and read_excel
</commit_message>
<xml_diff>
--- a/data/list_of_banks_ref.xlsx
+++ b/data/list_of_banks_ref.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="191">
   <si>
     <t>bank_name</t>
   </si>
@@ -153,12 +153,6 @@
     <t>has a good comparison table, information is very complete</t>
   </si>
   <si>
-    <t>https://www.argenta.be/fr/epargner/compte-d-epargne/compte-d-accroissement.html;
-https://www.argenta.be/fr/epargner/compte-d-epargne/compte-de-fidelite.html;
-https://www.argenta.be/fr/epargner/compte-d-epargne/e-epargne.html;
-https://www.argenta.be/fr/epargner/compte-d-epargne/compte-maxi.html;</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -185,6 +179,12 @@
   </si>
   <si>
     <t>The pdf source links are duplicates from the individual products links.</t>
+  </si>
+  <si>
+    <t>https://www.argenta.be/fr/epargner/compte-d-epargne/compte-d-accroissement.html;
+https://www.argenta.be/fr/epargner/compte-d-epargne/compte-de-fidelite.html;
+https://www.argenta.be/fr/epargner/compte-d-epargne/e-epargne.html;
+https://www.argenta.be/fr/epargner/compte-d-epargne/compte-maxi.html;</t>
   </si>
   <si>
     <r>
@@ -1944,7 +1944,7 @@
     <col customWidth="1" min="21" max="21" width="43.14"/>
     <col customWidth="1" min="22" max="22" width="10.14"/>
     <col customWidth="1" min="23" max="23" width="38.0"/>
-    <col customWidth="1" min="24" max="24" width="33.29"/>
+    <col customWidth="1" min="24" max="24" width="53.14"/>
     <col customWidth="1" min="25" max="25" width="26.29"/>
     <col customWidth="1" min="26" max="26" width="40.57"/>
     <col customWidth="1" min="27" max="27" width="10.57"/>
@@ -2068,7 +2068,7 @@
       <c r="AS1" s="14"/>
       <c r="AT1" s="15"/>
     </row>
-    <row r="2" ht="87.75" customHeight="1">
+    <row r="2" ht="203.25" customHeight="1">
       <c r="A2" s="16" t="s">
         <v>32</v>
       </c>
@@ -2114,24 +2114,22 @@
       <c r="Q2" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="R2" s="24" t="s">
+      <c r="R2" s="24"/>
+      <c r="S2" s="30" t="s">
         <v>44</v>
-      </c>
-      <c r="S2" s="30" t="s">
-        <v>45</v>
       </c>
       <c r="T2" s="24"/>
       <c r="U2" s="31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V2" s="32">
         <v>5.0</v>
       </c>
       <c r="W2" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="X2" s="33" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="Y2" s="34"/>
       <c r="Z2" s="18" t="s">
@@ -4295,20 +4293,10 @@
       <c r="AT40" s="36"/>
     </row>
     <row r="41">
-      <c r="A41" s="55" t="s">
+      <c r="B41" s="55" t="s">
         <v>187</v>
       </c>
-      <c r="B41" s="50"/>
-      <c r="C41" s="56" t="s">
-        <v>188</v>
-      </c>
       <c r="D41" s="56"/>
-      <c r="E41" s="57" t="s">
-        <v>189</v>
-      </c>
-      <c r="F41" s="58" t="s">
-        <v>190</v>
-      </c>
       <c r="G41" s="35"/>
       <c r="H41" s="35"/>
       <c r="I41" s="41"/>
@@ -4351,7 +4339,9 @@
       <c r="AT41" s="36"/>
     </row>
     <row r="42">
-      <c r="B42" s="50"/>
+      <c r="B42" s="56" t="s">
+        <v>188</v>
+      </c>
       <c r="C42" s="35"/>
       <c r="D42" s="35"/>
       <c r="E42" s="35"/>
@@ -4398,7 +4388,9 @@
       <c r="AT42" s="36"/>
     </row>
     <row r="43">
-      <c r="B43" s="50"/>
+      <c r="B43" s="57" t="s">
+        <v>189</v>
+      </c>
       <c r="C43" s="35"/>
       <c r="D43" s="35"/>
       <c r="E43" s="35"/>
@@ -4445,7 +4437,9 @@
       <c r="AT43" s="36"/>
     </row>
     <row r="44">
-      <c r="B44" s="50"/>
+      <c r="B44" s="58" t="s">
+        <v>190</v>
+      </c>
       <c r="C44" s="35"/>
       <c r="D44" s="35"/>
       <c r="E44" s="35"/>

</xml_diff>